<commit_message>
Update Strategic Execution Dashboard, consolidated Masterfile, and .gitignore
</commit_message>
<xml_diff>
--- a/data/Strategic Execution Dashboard.xlsx
+++ b/data/Strategic Execution Dashboard.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30606"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://share.philips.com/sites/GlobalMoSMT-2023/Shared Documents/General/2026/Goals Alignment 2026/Strategic Execution 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3320" documentId="8_{9B9C04DA-ABE2-4E9B-9FCF-AA5C7C703189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5A4BA57-CBB5-43E3-A661-F181EB486104}"/>
+  <xr:revisionPtr revIDLastSave="3339" documentId="8_{9B9C04DA-ABE2-4E9B-9FCF-AA5C7C703189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{736A0B24-C905-4A14-9278-294C93D80D9F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{31EBE344-35EA-49FE-9828-AF06217AD86D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{31EBE344-35EA-49FE-9828-AF06217AD86D}"/>
   </bookViews>
   <sheets>
     <sheet name="Mastersheet" sheetId="5" r:id="rId1"/>
     <sheet name="AOP Critical" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -366,7 +366,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="143">
   <si>
     <t>Strategic Imperatives</t>
   </si>
@@ -498,6 +498,9 @@
     <t>Q2</t>
   </si>
   <si>
+    <t>Q3</t>
+  </si>
+  <si>
     <t xml:space="preserve">If reported Red then
 state Cause  </t>
   </si>
@@ -581,6 +584,13 @@
     <t>Increase contract penetration %</t>
   </si>
   <si>
+    <t>-0.8% delta Vs AOP. Excluding GRC 0.7% YoY improvement.  LATAM renewals improved ITM Sep. Expected turnaround is Q4 2026 (Dec)</t>
+  </si>
+  <si>
+    <t>1) Funnel focus actions driven across regions for renewals.
+2) Contract Funnel tracked 90 days before expiry for timely renewals.</t>
+  </si>
+  <si>
     <t>Adjusted EBITA %</t>
   </si>
   <si>
@@ -605,200 +615,13 @@
     <t>Mn</t>
   </si>
   <si>
+    <t>YTD Sept Productivity no's on track.Good Realization from E&amp;E savings of Pune and also a gap reduction of R&amp;D Budget YTD.</t>
+  </si>
+  <si>
     <t>Inventory MAT sales</t>
   </si>
   <si>
     <t>Inventory as a % MAT sales</t>
-  </si>
-  <si>
-    <t>Inventory as a % MAT sales KPI</t>
-  </si>
-  <si>
-    <t>NPI Schedule Adherence</t>
-  </si>
-  <si>
-    <t>Shivaraj G</t>
-  </si>
-  <si>
-    <t>Dhruv  Schedule Adherence</t>
-  </si>
-  <si>
-    <t>Implied Market Share Gain</t>
-  </si>
-  <si>
-    <t>Sarika P</t>
-  </si>
-  <si>
-    <t>Implied Market Share Gain (ITQ)</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>QTR</t>
-  </si>
-  <si>
-    <t>Win Rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Win Rate </t>
-  </si>
-  <si>
-    <t>(Philips OIT) / (Philips OIT + lost SFDC + not pursuing SFDC)</t>
-  </si>
-  <si>
-    <t>Implied Market Share Gain KPI</t>
-  </si>
-  <si>
-    <t>Order Intake Growth</t>
-  </si>
-  <si>
-    <t>OIT Growth % (EQ)</t>
-  </si>
-  <si>
-    <t>OIT (Equipment  + Service)</t>
-  </si>
-  <si>
-    <t>OIT Growth % (CS)</t>
-  </si>
-  <si>
-    <t>Comparable Sales</t>
-  </si>
-  <si>
-    <t>Monthly Sales recognized (EQ)</t>
-  </si>
-  <si>
-    <t>CSG % KPI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impact Index KPI </t>
-  </si>
-  <si>
-    <t>Lakshmi M</t>
-  </si>
-  <si>
-    <t>EES scores are out! It is a balanced story. We are better than H1 2025 but slightly worse than H2 2025</t>
-  </si>
-  <si>
-    <t>CS has hit it out of the park.Quality dipped from 100% but still highest, Marketing is holding but at low scores. R&amp;D has dropped some big numbers.</t>
-  </si>
-  <si>
-    <t>Employee Engagement KPI</t>
-  </si>
-  <si>
-    <t>HY</t>
-  </si>
-  <si>
-    <t>MoS Value Levers 2026 - 2028:</t>
-  </si>
-  <si>
-    <t>Value Levers</t>
-  </si>
-  <si>
-    <t>AOP
- 2026</t>
-  </si>
-  <si>
-    <t>AOP
- 2027</t>
-  </si>
-  <si>
-    <t>AOP
- 2028</t>
-  </si>
-  <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>Cost Of Non-Quality as % of Sales</t>
-  </si>
-  <si>
-    <t>Cost of FCO, Warranty, Obsolescence, Scrap and Rework.</t>
-  </si>
-  <si>
-    <t>Competitive Roadmap</t>
-  </si>
-  <si>
-    <t>Roadmap MS% delivery (NPI OIT)</t>
-  </si>
-  <si>
-    <t>Zenition 10 &amp; 30 OIT below Q2 AOP due NPIs and price pressure from GE &amp; Siemens</t>
-  </si>
-  <si>
-    <t>Focus on Philips IB opportunity through mapping and targeted promotions to improve win rate</t>
-  </si>
-  <si>
-    <t>(MS% delivered by roadmap)
-/ (MS% ambition) 
-over 5 year horizon</t>
-  </si>
-  <si>
-    <t>Vitality index</t>
-  </si>
-  <si>
-    <t>% of sales from MoS Innovation &lt; 3 years</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Improve Z10 &amp; Z30 competitiveness (sales training to counter competition) and bundling service at POS address price gap
-</t>
-  </si>
-  <si>
-    <t>I2M Value Creation</t>
-  </si>
-  <si>
-    <t>Development progress (per year, per quarter, %) X Incremental IGM</t>
-  </si>
-  <si>
-    <t>Development progress 
-(per year, per quarter, %) X Incremental IGM,( from business cases, M€ )</t>
-  </si>
-  <si>
-    <t>Cusotomer Focus</t>
-  </si>
-  <si>
-    <t>Services - Time To System Up (TTSU)</t>
-  </si>
-  <si>
-    <t>% of system down cases back up &lt;48hrs</t>
-  </si>
-  <si>
-    <t>Time To System Up &lt; 48h</t>
-  </si>
-  <si>
-    <t>Profitability - Margin Expansion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Driving profitability via margin expansion  </t>
-  </si>
-  <si>
-    <t>Focus on optimizing FCP, pricing, and product mix to drive margin expansion</t>
-  </si>
-  <si>
-    <t>YTD Sept Productivity no's on track.Good Realization from E&amp;E savings of Pune and also a gap reduction of R&amp;D Budget YTD.</t>
-  </si>
-  <si>
-    <t>EQ OIT YTD Sep lower by 0.2M, which is mainly coming by NAR -4.4M, EU -3.7M however Growth supported by over-drive +7.9M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current OOH does not support FY revnue plan. 
-OOH is 117 M agaist AOP of 141M .B&amp;B  24 M B&amp;B required to meet FY AOP.
-</t>
-  </si>
-  <si>
-    <t>Growth</t>
-  </si>
-  <si>
-    <t>Drive B&amp;B OIT 
-NAR : 5 M , EU: 8.5M , Growth : 7.6</t>
-  </si>
-  <si>
-    <t>1. NAR :AOP accelator program launched to improve OIT to rev conversion.
-2. EU : Demo  liquidation plan aligned toward Q4 to maximise OIT in Q3.
-3. Growth:  Namibia tender conversion in Q4
-4. UIEP : COE team to analyse the difference and accurate capturing in AOP 2027</t>
   </si>
   <si>
     <t xml:space="preserve">Market inventory : 7.7 M above AOP .
@@ -809,11 +632,191 @@
 </t>
   </si>
   <si>
-    <t>1) Funnel focus actions driven across regions for renewals.
-2) Contract Funnel tracked 90 days before expiry for timely renewals.</t>
-  </si>
-  <si>
-    <t>-0.8% delta Vs AOP. Excluding GRC 0.7% YoY improvement.  LATAM renewals improved ITM Sep. Expected turnaround is Q4 2026 (Dec)</t>
+    <t>1. NAR :AOP accelator program launched to improve OIT to rev conversion.
+2. EU : Demo  liquidation plan aligned toward Q4 to maximise OIT in Q3.
+3. Growth:  Namibia tender conversion in Q4
+4. UIEP : COE team to analyse the difference and accurate capturing in AOP 2027</t>
+  </si>
+  <si>
+    <t>Inventory as a % MAT sales KPI</t>
+  </si>
+  <si>
+    <t>NPI Schedule Adherence</t>
+  </si>
+  <si>
+    <t>Shivaraj G</t>
+  </si>
+  <si>
+    <t>Dhruv  Schedule Adherence</t>
+  </si>
+  <si>
+    <t>Implied Market Share Gain</t>
+  </si>
+  <si>
+    <t>Sarika P</t>
+  </si>
+  <si>
+    <t>Implied Market Share Gain (ITQ)</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>QTR</t>
+  </si>
+  <si>
+    <t>Win Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Win Rate </t>
+  </si>
+  <si>
+    <t>(Philips OIT) / (Philips OIT + lost SFDC + not pursuing SFDC)</t>
+  </si>
+  <si>
+    <t>Implied Market Share Gain KPI</t>
+  </si>
+  <si>
+    <t>Order Intake Growth</t>
+  </si>
+  <si>
+    <t>OIT Growth % (EQ)</t>
+  </si>
+  <si>
+    <t>EQ OIT YTD Sep lower by 0.2M, which is mainly coming by NAR -4.4M, EU -3.7M however Growth supported by over-drive +7.9M</t>
+  </si>
+  <si>
+    <t>OIT (Equipment  + Service)</t>
+  </si>
+  <si>
+    <t>OIT Growth % (CS)</t>
+  </si>
+  <si>
+    <t>Comparable Sales</t>
+  </si>
+  <si>
+    <t>Monthly Sales recognized (EQ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current OOH does not support FY revnue plan. 
+OOH is 117 M agaist AOP of 141M .B&amp;B  24 M B&amp;B required to meet FY AOP.
+</t>
+  </si>
+  <si>
+    <t>Drive B&amp;B OIT 
+NAR : 5 M , EU: 8.5M , Growth : 7.6</t>
+  </si>
+  <si>
+    <t>CSG % KPI</t>
+  </si>
+  <si>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impact Index KPI </t>
+  </si>
+  <si>
+    <t>Lakshmi M</t>
+  </si>
+  <si>
+    <t>EES scores are out! It is a balanced story. We are better than H1 2025 but slightly worse than H2 2025</t>
+  </si>
+  <si>
+    <t>CS has hit it out of the park.Quality dipped from 100% but still highest, Marketing is holding but at low scores. R&amp;D has dropped some big numbers.</t>
+  </si>
+  <si>
+    <t>Employee Engagement KPI</t>
+  </si>
+  <si>
+    <t>HY</t>
+  </si>
+  <si>
+    <t>MoS Value Levers 2026 - 2028:</t>
+  </si>
+  <si>
+    <t>Value Levers</t>
+  </si>
+  <si>
+    <t>AOP
+ 2026</t>
+  </si>
+  <si>
+    <t>AOP
+ 2027</t>
+  </si>
+  <si>
+    <t>AOP
+ 2028</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>Cost Of Non-Quality as % of Sales</t>
+  </si>
+  <si>
+    <t>Cost of FCO, Warranty, Obsolescence, Scrap and Rework.</t>
+  </si>
+  <si>
+    <t>Competitive Roadmap</t>
+  </si>
+  <si>
+    <t>Roadmap MS% delivery (NPI OIT)</t>
+  </si>
+  <si>
+    <t>Zenition 10 &amp; 30 OIT below Q2 AOP due NPIs and price pressure from GE &amp; Siemens</t>
+  </si>
+  <si>
+    <t>Focus on Philips IB opportunity through mapping and targeted promotions to improve win rate</t>
+  </si>
+  <si>
+    <t>(MS% delivered by roadmap)
+/ (MS% ambition) 
+over 5 year horizon</t>
+  </si>
+  <si>
+    <t>Vitality index</t>
+  </si>
+  <si>
+    <t>% of sales from MoS Innovation &lt; 3 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improve Z10 &amp; Z30 competitiveness (sales training to counter competition) and bundling service at POS address price gap
+</t>
+  </si>
+  <si>
+    <t>I2M Value Creation</t>
+  </si>
+  <si>
+    <t>Development progress (per year, per quarter, %) X Incremental IGM</t>
+  </si>
+  <si>
+    <t>Development progress 
+(per year, per quarter, %) X Incremental IGM,( from business cases, M€ )</t>
+  </si>
+  <si>
+    <t>Cusotomer Focus</t>
+  </si>
+  <si>
+    <t>Services - Time To System Up (TTSU)</t>
+  </si>
+  <si>
+    <t>% of system down cases back up &lt;48hrs</t>
+  </si>
+  <si>
+    <t>Time To System Up &lt; 48h</t>
+  </si>
+  <si>
+    <t>Profitability - Margin Expansion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driving profitability via margin expansion  </t>
+  </si>
+  <si>
+    <t>Focus on optimizing FCP, pricing, and product mix to drive margin expansion</t>
   </si>
 </sst>
 </file>
@@ -821,13 +824,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="mmm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="mmm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1313,7 +1316,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1324,14 +1327,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1361,84 +1364,84 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1457,13 +1460,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="15" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="15" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="14" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="14" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="16" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="9" fillId="16" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="14" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1500,21 +1503,21 @@
     <xf numFmtId="10" fontId="8" fillId="7" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="17" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1523,28 +1526,28 @@
     <xf numFmtId="10" fontId="8" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="7" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1553,10 +1556,10 @@
     <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1855,7 +1858,35 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1876,7 +1907,35 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDEDDF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1939,83 +1998,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFDEDDF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFDEDDF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFDA9694"/>
         </patternFill>
       </fill>
@@ -2038,111 +2020,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFDEDDF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFDEDDF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFDEDDF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2191,6 +2068,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
@@ -2199,6 +2090,118 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDA9694"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2227,6 +2230,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFDEDDF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2276,13 +2286,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFDA9694"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5181,29 +5184,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{247AD843-49A7-417E-9F24-86908363EFA2}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:V59"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.54296875" customWidth="1"/>
-    <col min="5" max="6" width="10.453125" customWidth="1"/>
-    <col min="7" max="7" width="13.81640625" customWidth="1"/>
-    <col min="9" max="9" width="11.54296875" customWidth="1"/>
-    <col min="10" max="10" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="55.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" customWidth="1"/>
+    <col min="5" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="16" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" ht="15.95">
       <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:22">
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:22">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -5271,7 +5274,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22">
       <c r="A5" t="str">
         <f>IF('AOP Critical'!B6="","",'AOP Critical'!B6)</f>
         <v>Complaint Closure</v>
@@ -5357,7 +5360,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22">
       <c r="A6" t="str">
         <f>IF('AOP Critical'!B6="","",'AOP Critical'!B6)</f>
         <v>Complaint Closure</v>
@@ -5443,7 +5446,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22">
       <c r="A7" t="str">
         <f>IF('AOP Critical'!B8="","",'AOP Critical'!B8)</f>
         <v>% of CAPA investgation</v>
@@ -5529,7 +5532,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22">
       <c r="A8" t="str">
         <f>IF('AOP Critical'!B8="","",'AOP Critical'!B8)</f>
         <v>% of CAPA investgation</v>
@@ -5615,7 +5618,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22">
       <c r="A9" t="str">
         <f>IF('AOP Critical'!B10="","",'AOP Critical'!B10)</f>
         <v xml:space="preserve"># of Corrections &amp; Removals </v>
@@ -5684,9 +5687,9 @@
         <f>IF('AOP Critical'!S10="","",'AOP Critical'!S10)</f>
         <v>1</v>
       </c>
-      <c r="S9" t="str">
+      <c r="S9">
         <f>IF('AOP Critical'!T10="","",'AOP Critical'!T10)</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="T9" t="str">
         <f>IF('AOP Critical'!U10="","",'AOP Critical'!U10)</f>
@@ -5701,7 +5704,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22">
       <c r="A10" t="str">
         <f>IF('AOP Critical'!B10="","",'AOP Critical'!B10)</f>
         <v xml:space="preserve"># of Corrections &amp; Removals </v>
@@ -5787,7 +5790,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22">
       <c r="A11" t="str">
         <f>IF('AOP Critical'!B41="","",'AOP Critical'!B41)</f>
         <v>Cost Of Non-Quality as % of Sales</v>
@@ -5873,7 +5876,7 @@
         <v>3.32E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22">
       <c r="A12" t="str">
         <f>IF('AOP Critical'!B41="","",'AOP Critical'!B41)</f>
         <v>Cost Of Non-Quality as % of Sales</v>
@@ -5959,12 +5962,12 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22">
       <c r="A13" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -6032,7 +6035,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22">
       <c r="A15" t="str">
         <f>IF('AOP Critical'!B12="","",'AOP Critical'!B12)</f>
         <v>Ontime In Full</v>
@@ -6122,7 +6125,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22">
       <c r="A16" t="str">
         <f>IF('AOP Critical'!B12="","",'AOP Critical'!B12)</f>
         <v>Ontime In Full</v>
@@ -6212,7 +6215,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22">
       <c r="A17" t="str">
         <f>IF('AOP Critical'!B14="","",'AOP Critical'!B14)</f>
         <v>Contract Penetration</v>
@@ -6302,7 +6305,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22">
       <c r="A18" t="str">
         <f>IF('AOP Critical'!B14="","",'AOP Critical'!B14)</f>
         <v>Contract Penetration</v>
@@ -6392,7 +6395,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22">
       <c r="A19" t="str">
         <f>IF('AOP Critical'!B49="","",'AOP Critical'!B49)</f>
         <v>Services - Time To System Up (TTSU)</v>
@@ -6482,7 +6485,7 @@
         <v>0.73999999999999966</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22">
       <c r="A20" t="str">
         <f>IF('AOP Critical'!B49="","",'AOP Critical'!B49)</f>
         <v>Services - Time To System Up (TTSU)</v>
@@ -6572,12 +6575,12 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22">
       <c r="A21" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -6645,7 +6648,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22">
       <c r="A23" t="str">
         <f>IF('AOP Critical'!B16="","",'AOP Critical'!B16)</f>
         <v>Adjusted EBITA %</v>
@@ -6735,7 +6738,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22">
       <c r="A24" t="str">
         <f>IF('AOP Critical'!B16="","",'AOP Critical'!B16)</f>
         <v>Adjusted EBITA %</v>
@@ -6825,7 +6828,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22">
       <c r="A25" t="str">
         <f>IF('AOP Critical'!B18="","",'AOP Critical'!B18)</f>
         <v>Productivity</v>
@@ -6915,7 +6918,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22">
       <c r="A26" t="str">
         <f>IF('AOP Critical'!B18="","",'AOP Critical'!B18)</f>
         <v>Productivity</v>
@@ -7005,7 +7008,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22">
       <c r="A27" t="str">
         <f>IF('AOP Critical'!B20="","",'AOP Critical'!B20)</f>
         <v>Inventory MAT sales</v>
@@ -7095,7 +7098,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22">
       <c r="A28" t="str">
         <f>IF('AOP Critical'!B20="","",'AOP Critical'!B20)</f>
         <v>Inventory MAT sales</v>
@@ -7185,7 +7188,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22">
       <c r="A29" t="str">
         <f>IF('AOP Critical'!B51="","",'AOP Critical'!B51)</f>
         <v>Profitability - Margin Expansion</v>
@@ -7275,7 +7278,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22">
       <c r="A30" t="str">
         <f>IF('AOP Critical'!B51="","",'AOP Critical'!B51)</f>
         <v>Profitability - Margin Expansion</v>
@@ -7365,12 +7368,12 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22">
       <c r="A31" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -7438,7 +7441,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:22">
       <c r="A33" t="str">
         <f>IF('AOP Critical'!B26="","",'AOP Critical'!B26)</f>
         <v xml:space="preserve">Win Rate </v>
@@ -7528,7 +7531,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:22">
       <c r="A34" t="str">
         <f>IF('AOP Critical'!B26="","",'AOP Critical'!B26)</f>
         <v xml:space="preserve">Win Rate </v>
@@ -7618,7 +7621,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:22">
       <c r="A35" t="str">
         <f>IF('AOP Critical'!B22="","",'AOP Critical'!B22)</f>
         <v>NPI Schedule Adherence</v>
@@ -7708,7 +7711,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:22">
       <c r="A36" t="str">
         <f>IF('AOP Critical'!B22="","",'AOP Critical'!B22)</f>
         <v>NPI Schedule Adherence</v>
@@ -7798,7 +7801,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:22">
       <c r="A37" t="str">
         <f>IF('AOP Critical'!B43="","",'AOP Critical'!B43)</f>
         <v>Competitive Roadmap</v>
@@ -7888,7 +7891,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:22">
       <c r="A38" t="str">
         <f>IF('AOP Critical'!B43="","",'AOP Critical'!B43)</f>
         <v>Competitive Roadmap</v>
@@ -7978,7 +7981,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:22">
       <c r="A39" t="str">
         <f>IF('AOP Critical'!B45="","",'AOP Critical'!B45)</f>
         <v>Vitality index</v>
@@ -8068,7 +8071,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22">
       <c r="A40" t="str">
         <f>IF('AOP Critical'!B45="","",'AOP Critical'!B45)</f>
         <v>Vitality index</v>
@@ -8158,7 +8161,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:22">
       <c r="A41" t="str">
         <f>IF('AOP Critical'!B47="","",'AOP Critical'!B47)</f>
         <v>I2M Value Creation</v>
@@ -8248,7 +8251,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:22">
       <c r="A42" t="str">
         <f>IF('AOP Critical'!B47="","",'AOP Critical'!B47)</f>
         <v>I2M Value Creation</v>
@@ -8338,12 +8341,12 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:22">
       <c r="A43" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:22">
       <c r="A44" t="s">
         <v>2</v>
       </c>
@@ -8411,7 +8414,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:22">
       <c r="A45" t="str">
         <f>IF('AOP Critical'!D28="","",'AOP Critical'!D28)</f>
         <v>OIT Growth % (EQ)</v>
@@ -8501,7 +8504,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:22">
       <c r="A46" t="str">
         <f>IF('AOP Critical'!D28="","",'AOP Critical'!D28)</f>
         <v>OIT Growth % (EQ)</v>
@@ -8591,7 +8594,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:22">
       <c r="A47" t="str">
         <f>IF('AOP Critical'!D30="","",'AOP Critical'!D30)</f>
         <v>OIT Growth % (CS)</v>
@@ -8678,7 +8681,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:22">
       <c r="A48" t="str">
         <f>IF('AOP Critical'!D30="","",'AOP Critical'!D30)</f>
         <v>OIT Growth % (CS)</v>
@@ -8764,7 +8767,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:22">
       <c r="A49" t="str">
         <f>IF('AOP Critical'!B32="","",'AOP Critical'!B32)</f>
         <v>Comparable Sales</v>
@@ -8854,7 +8857,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:22">
       <c r="A50" t="str">
         <f>IF('AOP Critical'!B32="","",'AOP Critical'!B32)</f>
         <v>Comparable Sales</v>
@@ -8944,7 +8947,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:22">
       <c r="A51" t="str">
         <f>IF('AOP Critical'!B24="","",'AOP Critical'!B24)</f>
         <v>Implied Market Share Gain</v>
@@ -9019,7 +9022,7 @@
       </c>
       <c r="S51" s="70" t="str">
         <f>IF('AOP Critical'!T24="","",'AOP Critical'!T24)</f>
-        <v/>
+        <v>QTR</v>
       </c>
       <c r="T51" s="70" t="str">
         <f>IF('AOP Critical'!U24="","",'AOP Critical'!U24)</f>
@@ -9034,7 +9037,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:22">
       <c r="A52" t="str">
         <f>IF('AOP Critical'!B24="","",'AOP Critical'!B24)</f>
         <v>Implied Market Share Gain</v>
@@ -9097,7 +9100,7 @@
       </c>
       <c r="P52">
         <f>IF('AOP Critical'!Q25="","",'AOP Critical'!Q25)</f>
-        <v>0.121</v>
+        <v>0.12</v>
       </c>
       <c r="Q52" t="str">
         <f>IF('AOP Critical'!R25="","",'AOP Critical'!R25)</f>
@@ -9109,7 +9112,7 @@
       </c>
       <c r="S52" t="str">
         <f>IF('AOP Critical'!T25="","",'AOP Critical'!T25)</f>
-        <v/>
+        <v>QTR</v>
       </c>
       <c r="T52" t="str">
         <f>IF('AOP Critical'!U25="","",'AOP Critical'!U25)</f>
@@ -9124,12 +9127,12 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:22">
       <c r="A54" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:22">
       <c r="A55" t="s">
         <v>2</v>
       </c>
@@ -9197,7 +9200,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:22">
       <c r="A56" t="s">
         <v>29</v>
       </c>
@@ -9272,7 +9275,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:22">
       <c r="A57" t="s">
         <v>29</v>
       </c>
@@ -9347,7 +9350,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:22">
       <c r="A58" t="s">
         <v>35</v>
       </c>
@@ -9422,7 +9425,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:22">
       <c r="A59" t="s">
         <v>35</v>
       </c>
@@ -9482,7 +9485,7 @@
       </c>
       <c r="S59" s="69" t="str">
         <f>IF('AOP Critical'!T37="","",'AOP Critical'!T37)</f>
-        <v/>
+        <v>HY</v>
       </c>
       <c r="T59" s="69" t="str">
         <f>IF('AOP Critical'!U37="","",'AOP Critical'!U37)</f>
@@ -9518,34 +9521,35 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632542D1-52E6-4116-B536-B17D5839DF19}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AC52"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="20.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.45" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" customWidth="1"/>
-    <col min="2" max="2" width="27.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="26.81640625" customWidth="1"/>
-    <col min="5" max="5" width="5.1796875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="4.54296875" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="1.81640625" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="2.7265625" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.7265625" customWidth="1"/>
-    <col min="12" max="12" width="5.54296875" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="6.81640625" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="6.26953125" customWidth="1"/>
-    <col min="15" max="15" width="7.26953125" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="6.1796875" hidden="1" customWidth="1"/>
-    <col min="17" max="22" width="6.1796875" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="1.85546875" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" customWidth="1"/>
+    <col min="12" max="12" width="5.5703125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="6.85546875" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="6.28515625" customWidth="1"/>
+    <col min="15" max="15" width="7.28515625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="6.140625" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="22" width="6.140625" customWidth="1"/>
     <col min="23" max="23" width="6" customWidth="1"/>
-    <col min="24" max="24" width="58.81640625" style="20" customWidth="1"/>
-    <col min="25" max="25" width="68.1796875" customWidth="1"/>
-    <col min="26" max="26" width="17.7265625" customWidth="1"/>
+    <col min="24" max="24" width="58.85546875" style="20" customWidth="1"/>
+    <col min="25" max="25" width="68.140625" customWidth="1"/>
+    <col min="26" max="26" width="17.7109375" customWidth="1"/>
     <col min="27" max="27" width="57" style="13" customWidth="1"/>
-    <col min="28" max="46" width="8.54296875" customWidth="1"/>
+    <col min="28" max="46" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" ht="20.45" customHeight="1">
       <c r="B1" s="3" t="s">
         <v>39</v>
       </c>
@@ -9556,7 +9560,7 @@
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" ht="20.45" customHeight="1">
       <c r="B2" s="6"/>
       <c r="C2" s="7"/>
       <c r="E2" s="6"/>
@@ -9565,7 +9569,7 @@
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
     </row>
-    <row r="3" spans="1:27" s="5" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="5" customFormat="1" ht="20.45" customHeight="1">
       <c r="A3" s="110" t="s">
         <v>40</v>
       </c>
@@ -9589,7 +9593,7 @@
       <c r="X3" s="89"/>
       <c r="AA3" s="14"/>
     </row>
-    <row r="4" spans="1:27" s="5" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="5" customFormat="1" ht="20.45" customHeight="1">
       <c r="A4" s="112" t="str">
         <f ca="1">"Current Month-Year " &amp; ":" &amp; TEXT(TODAY(),"YYYY-MM")</f>
         <v>Current Month-Year :2026-10</v>
@@ -9621,7 +9625,7 @@
       <c r="Z4" s="112"/>
       <c r="AA4" s="112"/>
     </row>
-    <row r="5" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" ht="20.45" customHeight="1">
       <c r="A5" s="85" t="s">
         <v>0</v>
       </c>
@@ -9676,7 +9680,7 @@
         <v>19</v>
       </c>
       <c r="T5" s="34" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="U5" s="34" t="s">
         <v>21</v>
@@ -9688,30 +9692,30 @@
         <v>23</v>
       </c>
       <c r="X5" s="23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y5" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Z5" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA5" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" ht="14.45">
       <c r="A6" s="109" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="91" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="92" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D6" s="90" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E6" s="108">
         <v>10</v>
@@ -9719,16 +9723,16 @@
       <c r="F6" s="108"/>
       <c r="G6" s="108"/>
       <c r="H6" s="111" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I6" s="108" t="s">
         <v>33</v>
       </c>
       <c r="J6" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L6" s="35">
         <v>0.08</v>
@@ -9770,10 +9774,10 @@
       <c r="Y6" s="113"/>
       <c r="Z6" s="113"/>
       <c r="AA6" s="123" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27" ht="14.45">
       <c r="A7" s="109"/>
       <c r="B7" s="91"/>
       <c r="C7" s="92"/>
@@ -9785,7 +9789,7 @@
       <c r="I7" s="108"/>
       <c r="J7" s="107"/>
       <c r="K7" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L7" s="17">
         <v>3.7999999999999999E-2</v>
@@ -9822,16 +9826,16 @@
       <c r="Z7" s="96"/>
       <c r="AA7" s="124"/>
     </row>
-    <row r="8" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" ht="14.45">
       <c r="A8" s="109"/>
       <c r="B8" s="91" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C8" s="92" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" s="90" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E8" s="108">
         <v>90</v>
@@ -9845,10 +9849,10 @@
         <v>33</v>
       </c>
       <c r="J8" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K8" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L8" s="35">
         <v>0.9</v>
@@ -9880,10 +9884,10 @@
       <c r="Y8" s="95"/>
       <c r="Z8" s="114"/>
       <c r="AA8" s="123" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" ht="14.45">
       <c r="A9" s="109"/>
       <c r="B9" s="91"/>
       <c r="C9" s="92"/>
@@ -9895,7 +9899,7 @@
       <c r="I9" s="108"/>
       <c r="J9" s="107"/>
       <c r="K9" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L9" s="19">
         <v>1</v>
@@ -9932,16 +9936,16 @@
       <c r="Z9" s="115"/>
       <c r="AA9" s="124"/>
     </row>
-    <row r="10" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" ht="14.45">
       <c r="A10" s="109"/>
       <c r="B10" s="91" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" s="92" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="90" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E10" s="108">
         <v>1</v>
@@ -9949,16 +9953,16 @@
       <c r="F10" s="108"/>
       <c r="G10" s="108"/>
       <c r="H10" s="111" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I10" s="108" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J10" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K10" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L10" s="36">
         <v>1</v>
@@ -9984,7 +9988,9 @@
       <c r="S10" s="8">
         <v>1</v>
       </c>
-      <c r="T10" s="8"/>
+      <c r="T10" s="8">
+        <v>1</v>
+      </c>
       <c r="U10" s="8"/>
       <c r="V10" s="8"/>
       <c r="W10" s="33"/>
@@ -9992,10 +9998,10 @@
       <c r="Y10" s="164"/>
       <c r="Z10" s="117"/>
       <c r="AA10" s="123" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:27" ht="15" thickBot="1">
       <c r="A11" s="109"/>
       <c r="B11" s="91"/>
       <c r="C11" s="92"/>
@@ -10007,7 +10013,7 @@
       <c r="I11" s="108"/>
       <c r="J11" s="107"/>
       <c r="K11" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L11" s="9">
         <v>2</v>
@@ -10044,18 +10050,18 @@
       <c r="Z11" s="118"/>
       <c r="AA11" s="124"/>
     </row>
-    <row r="12" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27" ht="14.45">
       <c r="A12" s="109" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="93" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" s="93" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12" s="90" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E12" s="108">
         <v>84</v>
@@ -10069,10 +10075,10 @@
         <v>33</v>
       </c>
       <c r="J12" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K12" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L12" s="35">
         <v>0.69</v>
@@ -10114,10 +10120,10 @@
       <c r="Y12" s="95"/>
       <c r="Z12" s="96"/>
       <c r="AA12" s="123" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:27" ht="14.45">
       <c r="A13" s="109"/>
       <c r="B13" s="93"/>
       <c r="C13" s="93"/>
@@ -10129,7 +10135,7 @@
       <c r="I13" s="108"/>
       <c r="J13" s="107"/>
       <c r="K13" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L13" s="19">
         <v>0.83</v>
@@ -10166,16 +10172,16 @@
       <c r="Z13" s="96"/>
       <c r="AA13" s="124"/>
     </row>
-    <row r="14" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27" ht="14.45">
       <c r="A14" s="109"/>
       <c r="B14" s="93" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" s="122" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="90" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="108">
         <v>54.6</v>
@@ -10189,10 +10195,10 @@
         <v>33</v>
       </c>
       <c r="J14" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K14" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L14" s="37">
         <v>0.54249999999999998</v>
@@ -10225,15 +10231,15 @@
       <c r="V14" s="37"/>
       <c r="W14" s="37"/>
       <c r="X14" s="152" t="s">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="Y14" s="97" t="s">
-        <v>140</v>
+        <v>72</v>
       </c>
       <c r="Z14" s="154"/>
       <c r="AA14" s="151"/>
     </row>
-    <row r="15" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:27" ht="15" thickBot="1">
       <c r="A15" s="109"/>
       <c r="B15" s="93"/>
       <c r="C15" s="122"/>
@@ -10245,7 +10251,7 @@
       <c r="I15" s="108"/>
       <c r="J15" s="107"/>
       <c r="K15" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L15" s="17">
         <v>0.51780000000000004</v>
@@ -10282,21 +10288,21 @@
       <c r="Z15" s="113"/>
       <c r="AA15" s="131"/>
     </row>
-    <row r="16" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" ht="14.45">
       <c r="A16" s="109" t="s">
         <v>25</v>
       </c>
       <c r="B16" s="93" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C16" s="93" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D16" s="90" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E16" s="108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F16" s="108"/>
       <c r="G16" s="108"/>
@@ -10307,10 +10313,10 @@
         <v>33</v>
       </c>
       <c r="J16" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K16" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L16" s="37">
         <v>0.11774014693384624</v>
@@ -10346,10 +10352,10 @@
       <c r="Y16" s="95"/>
       <c r="Z16" s="115"/>
       <c r="AA16" s="123" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:27" ht="14.45">
       <c r="A17" s="109"/>
       <c r="B17" s="93"/>
       <c r="C17" s="93"/>
@@ -10361,7 +10367,7 @@
       <c r="I17" s="108"/>
       <c r="J17" s="107"/>
       <c r="K17" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L17" s="17">
         <v>-4.253311543933095E-2</v>
@@ -10398,19 +10404,19 @@
       <c r="Z17" s="115"/>
       <c r="AA17" s="124"/>
     </row>
-    <row r="18" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" ht="14.45">
       <c r="A18" s="109"/>
       <c r="B18" s="93" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C18" s="93" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D18" s="93" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="108" t="s">
         <v>76</v>
-      </c>
-      <c r="E18" s="108" t="s">
-        <v>73</v>
       </c>
       <c r="F18" s="108"/>
       <c r="G18" s="108"/>
@@ -10418,13 +10424,13 @@
         <v>32</v>
       </c>
       <c r="I18" s="108" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J18" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K18" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L18" s="47">
         <v>0.224</v>
@@ -10457,7 +10463,7 @@
       <c r="V18" s="47"/>
       <c r="W18" s="47"/>
       <c r="X18" s="158" t="s">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="Y18" s="158"/>
       <c r="Z18" s="155">
@@ -10465,7 +10471,7 @@
       </c>
       <c r="AA18" s="157"/>
     </row>
-    <row r="19" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" ht="14.45">
       <c r="A19" s="109"/>
       <c r="B19" s="93"/>
       <c r="C19" s="93"/>
@@ -10477,7 +10483,7 @@
       <c r="I19" s="108"/>
       <c r="J19" s="107"/>
       <c r="K19" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L19" s="87">
         <v>0.2598381666666667</v>
@@ -10514,33 +10520,33 @@
       <c r="Z19" s="156"/>
       <c r="AA19" s="157"/>
     </row>
-    <row r="20" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:27" ht="14.45">
       <c r="A20" s="109"/>
       <c r="B20" s="93" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C20" s="93" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" s="90" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E20" s="108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F20" s="108"/>
       <c r="G20" s="108"/>
       <c r="H20" s="111" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I20" s="108" t="s">
         <v>33</v>
       </c>
       <c r="J20" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K20" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L20" s="35">
         <v>0.28399999999999997</v>
@@ -10573,17 +10579,17 @@
       <c r="V20" s="18"/>
       <c r="W20" s="27"/>
       <c r="X20" s="99" t="s">
-        <v>139</v>
+        <v>84</v>
       </c>
       <c r="Y20" s="101" t="s">
-        <v>138</v>
+        <v>85</v>
       </c>
       <c r="Z20" s="153"/>
       <c r="AA20" s="125" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:27" ht="15" thickBot="1">
       <c r="A21" s="109"/>
       <c r="B21" s="93"/>
       <c r="C21" s="93"/>
@@ -10595,7 +10601,7 @@
       <c r="I21" s="108"/>
       <c r="J21" s="107"/>
       <c r="K21" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L21" s="19">
         <v>0.27400000000000002</v>
@@ -10632,18 +10638,18 @@
       <c r="Z21" s="119"/>
       <c r="AA21" s="125"/>
     </row>
-    <row r="22" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:27" ht="14.45">
       <c r="A22" s="109" t="s">
         <v>26</v>
       </c>
       <c r="B22" s="93" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C22" s="122" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D22" s="93" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E22" s="108">
         <v>90</v>
@@ -10657,10 +10663,10 @@
         <v>33</v>
       </c>
       <c r="J22" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K22" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L22" s="35">
         <v>0.9</v>
@@ -10705,7 +10711,7 @@
       </c>
       <c r="AA22" s="162"/>
     </row>
-    <row r="23" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:27" ht="15" thickBot="1">
       <c r="A23" s="169"/>
       <c r="B23" s="93"/>
       <c r="C23" s="122"/>
@@ -10717,7 +10723,7 @@
       <c r="I23" s="108"/>
       <c r="J23" s="107"/>
       <c r="K23" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L23" s="54">
         <v>0.81</v>
@@ -10725,25 +10731,25 @@
       <c r="M23" s="54">
         <v>0.78</v>
       </c>
-      <c r="N23" s="19">
+      <c r="N23" s="56">
         <v>0.8</v>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="56">
         <v>0.82</v>
       </c>
-      <c r="P23" s="19">
+      <c r="P23" s="56">
         <v>0.79500000000000004</v>
       </c>
-      <c r="Q23" s="19">
+      <c r="Q23" s="56">
         <v>0.86</v>
       </c>
-      <c r="R23" s="29">
+      <c r="R23" s="56">
         <v>0.88</v>
       </c>
-      <c r="S23" s="29">
+      <c r="S23" s="56">
         <v>0.94</v>
       </c>
-      <c r="T23" s="29">
+      <c r="T23" s="56">
         <v>0.94</v>
       </c>
       <c r="U23" s="29"/>
@@ -10754,27 +10760,27 @@
       <c r="Z23" s="115"/>
       <c r="AA23" s="163"/>
     </row>
-    <row r="24" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" ht="14.45">
       <c r="A24" s="143" t="s">
         <v>27</v>
       </c>
       <c r="B24" s="93" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C24" s="122" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D24" s="90" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E24" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F24" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G24" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H24" s="111" t="s">
         <v>32</v>
@@ -10786,7 +10792,7 @@
         <v>34</v>
       </c>
       <c r="K24" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L24" s="35"/>
       <c r="M24" s="35"/>
@@ -10794,21 +10800,23 @@
         <v>0.104</v>
       </c>
       <c r="O24" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="P24" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q24" s="37">
         <v>0.11799999999999999</v>
       </c>
       <c r="R24" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="S24" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="T24" s="35"/>
+        <v>94</v>
+      </c>
+      <c r="T24" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="U24" s="21"/>
       <c r="V24" s="21"/>
       <c r="W24" s="38"/>
@@ -10816,10 +10824,10 @@
       <c r="Y24" s="154"/>
       <c r="Z24" s="119"/>
       <c r="AA24" s="123" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:27" ht="15" thickBot="1">
       <c r="A25" s="168"/>
       <c r="B25" s="93"/>
       <c r="C25" s="122"/>
@@ -10831,33 +10839,35 @@
       <c r="I25" s="108"/>
       <c r="J25" s="120"/>
       <c r="K25" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L25" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="M25" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="N25" s="50">
         <v>0.115</v>
       </c>
       <c r="O25" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="P25" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q25" s="17">
-        <v>0.121</v>
+        <v>0.12</v>
       </c>
       <c r="R25" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="S25" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="T25" s="55"/>
+        <v>94</v>
+      </c>
+      <c r="T25" s="21" t="s">
+        <v>94</v>
+      </c>
       <c r="U25" s="21"/>
       <c r="V25" s="21"/>
       <c r="W25" s="55"/>
@@ -10866,16 +10876,16 @@
       <c r="Z25" s="153"/>
       <c r="AA25" s="124"/>
     </row>
-    <row r="26" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" ht="14.45">
       <c r="A26" s="168"/>
       <c r="B26" s="91" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C26" s="161" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D26" s="90" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E26" s="108">
         <v>34</v>
@@ -10889,10 +10899,10 @@
         <v>33</v>
       </c>
       <c r="J26" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K26" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L26" s="35">
         <v>0.34</v>
@@ -10900,25 +10910,25 @@
       <c r="M26" s="35">
         <v>0.34</v>
       </c>
-      <c r="N26" s="35">
+      <c r="N26" s="18">
         <v>0.34</v>
       </c>
-      <c r="O26" s="35">
+      <c r="O26" s="18">
         <v>0.34</v>
       </c>
-      <c r="P26" s="35">
+      <c r="P26" s="18">
         <v>0.34</v>
       </c>
-      <c r="Q26" s="35">
+      <c r="Q26" s="18">
         <v>0.34</v>
       </c>
-      <c r="R26" s="35">
+      <c r="R26" s="18">
         <v>0.34</v>
       </c>
-      <c r="S26" s="24">
+      <c r="S26" s="18">
         <v>0.34</v>
       </c>
-      <c r="T26" s="24">
+      <c r="T26" s="18">
         <v>0.34</v>
       </c>
       <c r="U26" s="24"/>
@@ -10928,10 +10938,10 @@
       <c r="Y26" s="96"/>
       <c r="Z26" s="115"/>
       <c r="AA26" s="123" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:27" ht="15" thickBot="1">
       <c r="A27" s="168"/>
       <c r="B27" s="91"/>
       <c r="C27" s="161"/>
@@ -10943,7 +10953,7 @@
       <c r="I27" s="108"/>
       <c r="J27" s="107"/>
       <c r="K27" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L27" s="78">
         <v>0.318</v>
@@ -10980,19 +10990,19 @@
       <c r="Z27" s="115"/>
       <c r="AA27" s="124"/>
     </row>
-    <row r="28" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" ht="14.45">
       <c r="A28" s="168"/>
       <c r="B28" s="90" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C28" s="93" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D28" s="90" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E28" s="108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F28" s="108"/>
       <c r="G28" s="108"/>
@@ -11003,10 +11013,10 @@
         <v>33</v>
       </c>
       <c r="J28" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K28" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L28" s="37" vm="1">
         <v>3.6951550944796852E-2</v>
@@ -11039,15 +11049,15 @@
       <c r="V28" s="24"/>
       <c r="W28" s="25"/>
       <c r="X28" s="103" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="Y28" s="97"/>
       <c r="Z28" s="119"/>
       <c r="AA28" s="128" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:27" ht="15" thickBot="1">
       <c r="A29" s="168"/>
       <c r="B29" s="90"/>
       <c r="C29" s="93"/>
@@ -11059,7 +11069,7 @@
       <c r="I29" s="108"/>
       <c r="J29" s="107"/>
       <c r="K29" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L29" s="17" vm="2">
         <v>-0.21537837470975407</v>
@@ -11096,17 +11106,17 @@
       <c r="Z29" s="153"/>
       <c r="AA29" s="129"/>
     </row>
-    <row r="30" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:27" ht="14.45">
       <c r="A30" s="168"/>
       <c r="B30" s="90"/>
       <c r="C30" s="93" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D30" s="90" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E30" s="108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F30" s="108"/>
       <c r="G30" s="108"/>
@@ -11117,10 +11127,10 @@
         <v>33</v>
       </c>
       <c r="J30" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K30" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L30" s="37">
         <v>0.35899999999999999</v>
@@ -11157,7 +11167,7 @@
       <c r="Z30" s="119"/>
       <c r="AA30" s="166"/>
     </row>
-    <row r="31" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:27" ht="14.45">
       <c r="A31" s="168"/>
       <c r="B31" s="90"/>
       <c r="C31" s="93"/>
@@ -11169,7 +11179,7 @@
       <c r="I31" s="108"/>
       <c r="J31" s="107"/>
       <c r="K31" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L31" s="17">
         <v>0.32500000000000001</v>
@@ -11206,19 +11216,19 @@
       <c r="Z31" s="153"/>
       <c r="AA31" s="167"/>
     </row>
-    <row r="32" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" ht="14.45">
       <c r="A32" s="168"/>
       <c r="B32" s="93" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C32" s="122" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D32" s="90" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E32" s="108" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F32" s="108"/>
       <c r="G32" s="108"/>
@@ -11226,13 +11236,13 @@
         <v>32</v>
       </c>
       <c r="I32" s="108" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J32" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K32" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L32" s="41">
         <v>8.6903037999999988</v>
@@ -11265,17 +11275,17 @@
       <c r="V32" s="8"/>
       <c r="W32" s="33"/>
       <c r="X32" s="170" t="s">
-        <v>135</v>
+        <v>106</v>
       </c>
       <c r="Y32" s="97" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="Z32" s="119"/>
       <c r="AA32" s="123" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
     </row>
-    <row r="33" spans="1:29" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:29" ht="15" thickBot="1">
       <c r="A33" s="168"/>
       <c r="B33" s="93"/>
       <c r="C33" s="122"/>
@@ -11287,7 +11297,7 @@
       <c r="I33" s="108"/>
       <c r="J33" s="107"/>
       <c r="K33" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L33" s="42">
         <v>4.05</v>
@@ -11324,7 +11334,7 @@
       <c r="Z33" s="153"/>
       <c r="AA33" s="124"/>
     </row>
-    <row r="34" spans="1:29" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:29" ht="14.45">
       <c r="A34" s="109" t="s">
         <v>28</v>
       </c>
@@ -11332,7 +11342,7 @@
         <v>29</v>
       </c>
       <c r="C34" s="93" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D34" s="90" t="s">
         <v>31</v>
@@ -11352,7 +11362,7 @@
         <v>34</v>
       </c>
       <c r="K34" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L34" s="35"/>
       <c r="M34" s="35"/>
@@ -11376,14 +11386,14 @@
       </c>
       <c r="X34" s="94"/>
       <c r="Y34" s="96" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="Z34" s="115"/>
       <c r="AA34" s="123" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
-    <row r="35" spans="1:29" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:29" ht="14.45">
       <c r="A35" s="109"/>
       <c r="B35" s="148"/>
       <c r="C35" s="93"/>
@@ -11395,31 +11405,31 @@
       <c r="I35" s="108"/>
       <c r="J35" s="120"/>
       <c r="K35" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="M35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="N35" s="19">
         <v>1</v>
       </c>
       <c r="O35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="P35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q35" s="19">
         <v>0.96199999999999997</v>
       </c>
       <c r="R35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="S35" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="T35" s="19">
         <v>0.91300000000000003</v>
@@ -11432,13 +11442,13 @@
       <c r="Z35" s="115"/>
       <c r="AA35" s="124"/>
     </row>
-    <row r="36" spans="1:29" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:29" ht="14.45">
       <c r="A36" s="109"/>
       <c r="B36" s="148" t="s">
         <v>35</v>
       </c>
       <c r="C36" s="93" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D36" s="90" t="s">
         <v>37</v>
@@ -11458,7 +11468,7 @@
         <v>38</v>
       </c>
       <c r="K36" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L36" s="35"/>
       <c r="M36" s="35"/>
@@ -11477,17 +11487,17 @@
       <c r="V36" s="18"/>
       <c r="W36" s="27"/>
       <c r="X36" s="94" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="Y36" s="95" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="Z36" s="115"/>
       <c r="AA36" s="123" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="37" spans="1:29" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:29" ht="14.45">
       <c r="A37" s="109"/>
       <c r="B37" s="148"/>
       <c r="C37" s="93"/>
@@ -11499,31 +11509,33 @@
       <c r="I37" s="108"/>
       <c r="J37" s="121"/>
       <c r="K37" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L37" s="21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="M37" s="21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N37" s="21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="O37" s="19">
         <v>0.79</v>
       </c>
       <c r="P37" s="21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="Q37" s="19">
         <v>0.79</v>
       </c>
       <c r="R37" s="21" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="S37" s="56"/>
-      <c r="T37" s="56"/>
+      <c r="T37" s="21" t="s">
+        <v>115</v>
+      </c>
       <c r="U37" s="56"/>
       <c r="V37" s="56"/>
       <c r="W37" s="57"/>
@@ -11532,7 +11544,7 @@
       <c r="Z37" s="119"/>
       <c r="AA37" s="125"/>
     </row>
-    <row r="38" spans="1:29" s="5" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:29" s="5" customFormat="1" ht="20.45" customHeight="1">
       <c r="A38" s="138"/>
       <c r="B38" s="138"/>
       <c r="C38" s="138"/>
@@ -11561,9 +11573,9 @@
       <c r="Z38" s="139"/>
       <c r="AA38" s="139"/>
     </row>
-    <row r="39" spans="1:29" s="5" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:29" s="5" customFormat="1" ht="20.45" customHeight="1">
       <c r="A39" s="141" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B39" s="141"/>
       <c r="C39" s="58"/>
@@ -11592,12 +11604,12 @@
       <c r="Z39"/>
       <c r="AA39" s="13"/>
     </row>
-    <row r="40" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:29" ht="20.45" customHeight="1">
       <c r="A40" s="43" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C40" s="10" t="s">
         <v>3</v>
@@ -11606,13 +11618,13 @@
         <v>4</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="H40" s="10" t="s">
         <v>8</v>
@@ -11633,7 +11645,7 @@
         <v>13</v>
       </c>
       <c r="N40" s="10" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="O40" s="10" t="s">
         <v>15</v>
@@ -11642,7 +11654,7 @@
         <v>16</v>
       </c>
       <c r="Q40" s="10" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="R40" s="10" t="s">
         <v>18</v>
@@ -11663,51 +11675,51 @@
         <v>23</v>
       </c>
       <c r="X40" s="60" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y40" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Z40" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA40" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:29" ht="20.45" customHeight="1">
       <c r="A41" s="142" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B41" s="145" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="C41" s="146" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D41" s="147" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="E41" s="140" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F41" s="140" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G41" s="140" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H41" s="160" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I41" s="140" t="s">
         <v>33</v>
       </c>
       <c r="J41" s="149" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K41" s="61" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L41" s="76">
         <v>1.9099999999999999E-2</v>
@@ -11749,11 +11761,11 @@
       <c r="Y41" s="131"/>
       <c r="Z41" s="131"/>
       <c r="AA41" s="124" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="AC41" s="12"/>
     </row>
-    <row r="42" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:29" ht="20.45" customHeight="1">
       <c r="A42" s="143"/>
       <c r="B42" s="91"/>
       <c r="C42" s="92"/>
@@ -11765,7 +11777,7 @@
       <c r="I42" s="108"/>
       <c r="J42" s="127"/>
       <c r="K42" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L42" s="55">
         <v>9.1999999999999998E-3</v>
@@ -11802,27 +11814,27 @@
       <c r="Z42" s="131"/>
       <c r="AA42" s="126"/>
     </row>
-    <row r="43" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:29" ht="20.45" customHeight="1">
       <c r="A43" s="144" t="s">
         <v>26</v>
       </c>
       <c r="B43" s="91" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="C43" s="92" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D43" s="90" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="E43" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F43" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G43" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H43" s="111" t="s">
         <v>32</v>
@@ -11834,7 +11846,7 @@
         <v>34</v>
       </c>
       <c r="K43" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L43" s="35"/>
       <c r="M43" s="35"/>
@@ -11853,17 +11865,17 @@
       <c r="V43" s="35"/>
       <c r="W43" s="38"/>
       <c r="X43" s="130" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="Y43" s="132" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z43" s="133"/>
       <c r="AA43" s="134" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
-    <row r="44" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:29" ht="20.45" customHeight="1">
       <c r="A44" s="144"/>
       <c r="B44" s="91"/>
       <c r="C44" s="92"/>
@@ -11875,38 +11887,38 @@
       <c r="I44" s="159"/>
       <c r="J44" s="120"/>
       <c r="K44" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="M44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="N44" s="17">
         <v>4.2000000000000003E-2</v>
       </c>
       <c r="O44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="P44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="Q44" s="17">
         <v>0.04</v>
       </c>
       <c r="R44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="S44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="T44" s="55"/>
       <c r="U44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="V44" s="21" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="W44" s="55"/>
       <c r="X44" s="130"/>
@@ -11914,25 +11926,25 @@
       <c r="Z44" s="133"/>
       <c r="AA44" s="134"/>
     </row>
-    <row r="45" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:29" ht="20.45" customHeight="1">
       <c r="A45" s="144"/>
       <c r="B45" s="91" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C45" s="92" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D45" s="90" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="E45" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F45" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G45" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H45" s="111" t="s">
         <v>32</v>
@@ -11941,10 +11953,10 @@
         <v>33</v>
       </c>
       <c r="J45" s="127" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K45" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L45" s="35">
         <v>0.4</v>
@@ -11978,16 +11990,16 @@
       <c r="W45" s="38"/>
       <c r="X45" s="130"/>
       <c r="Y45" s="132" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="Z45" s="135">
         <v>46188</v>
       </c>
       <c r="AA45" s="126" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
-    <row r="46" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:29" ht="20.45" customHeight="1">
       <c r="A46" s="144"/>
       <c r="B46" s="91"/>
       <c r="C46" s="92"/>
@@ -11999,7 +12011,7 @@
       <c r="I46" s="108"/>
       <c r="J46" s="127"/>
       <c r="K46" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L46" s="19">
         <v>0.66</v>
@@ -12036,37 +12048,37 @@
       <c r="Z46" s="133"/>
       <c r="AA46" s="126"/>
     </row>
-    <row r="47" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:29" ht="20.45" customHeight="1">
       <c r="A47" s="144"/>
       <c r="B47" s="91" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="C47" s="92" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D47" s="90" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="E47" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F47" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G47" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H47" s="111" t="s">
         <v>32</v>
       </c>
       <c r="I47" s="108" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J47" s="127" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K47" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L47" s="36">
         <v>5.5</v>
@@ -12108,10 +12120,10 @@
       <c r="Y47" s="133"/>
       <c r="Z47" s="133"/>
       <c r="AA47" s="90" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
     </row>
-    <row r="48" spans="1:29" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:29" ht="20.45" customHeight="1">
       <c r="A48" s="144"/>
       <c r="B48" s="91"/>
       <c r="C48" s="92"/>
@@ -12123,7 +12135,7 @@
       <c r="I48" s="108"/>
       <c r="J48" s="127"/>
       <c r="K48" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L48" s="9">
         <v>9</v>
@@ -12161,27 +12173,27 @@
       <c r="Z48" s="133"/>
       <c r="AA48" s="90"/>
     </row>
-    <row r="49" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:27" ht="20.45" customHeight="1">
       <c r="A49" s="143" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="B49" s="150" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="C49" s="92" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D49" s="90" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E49" s="108">
         <v>74</v>
       </c>
       <c r="F49" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G49" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H49" s="111" t="s">
         <v>32</v>
@@ -12190,10 +12202,10 @@
         <v>33</v>
       </c>
       <c r="J49" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K49" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L49" s="37">
         <v>0.73199999999999998</v>
@@ -12235,10 +12247,10 @@
       <c r="Y49" s="132"/>
       <c r="Z49" s="133"/>
       <c r="AA49" s="126" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:27" ht="20.45" customHeight="1">
       <c r="A50" s="143"/>
       <c r="B50" s="150"/>
       <c r="C50" s="92"/>
@@ -12250,7 +12262,7 @@
       <c r="I50" s="108"/>
       <c r="J50" s="107"/>
       <c r="K50" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L50" s="17">
         <v>0.69299999999999995</v>
@@ -12287,27 +12299,27 @@
       <c r="Z50" s="133"/>
       <c r="AA50" s="126"/>
     </row>
-    <row r="51" spans="1:27" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:27" ht="20.45" customHeight="1">
       <c r="A51" s="144" t="s">
         <v>25</v>
       </c>
       <c r="B51" s="91" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="C51" s="92" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D51" s="90" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="E51" s="108">
         <v>33.1</v>
       </c>
       <c r="F51" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G51" s="108" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H51" s="111" t="s">
         <v>32</v>
@@ -12316,10 +12328,10 @@
         <v>33</v>
       </c>
       <c r="J51" s="107" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K51" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L51" s="37">
         <v>0.34700072985878605</v>
@@ -12355,10 +12367,10 @@
       <c r="Y51" s="133"/>
       <c r="Z51" s="133"/>
       <c r="AA51" s="93" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
     </row>
-    <row r="52" spans="1:27" ht="20.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:27" ht="20.45" customHeight="1" thickBot="1">
       <c r="A52" s="144"/>
       <c r="B52" s="91"/>
       <c r="C52" s="92"/>
@@ -12370,7 +12382,7 @@
       <c r="I52" s="108"/>
       <c r="J52" s="107"/>
       <c r="K52" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L52" s="17">
         <v>0.36591770011686803</v>
@@ -12727,34 +12739,34 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L27">
-    <cfRule type="expression" dxfId="66" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="66" priority="78">
+      <formula>AND(OR($H26="Lower the better", $H26="Lower the Better"), L27&gt;L26)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="79">
+      <formula>AND(OR($H26="Lower the better", $H26="Lower the Better"), L27&lt;=L26)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="80">
+      <formula>AND(OR($H26="Higher the better", $H26="Higher the Better"), L27&lt;L26)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="63" priority="81" stopIfTrue="1">
       <formula>AND(OR($H26="Higher the better", $H26="Higher the Better"), L27&gt;=L26)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="80">
-      <formula>AND(OR($H26="Higher the better", $H26="Higher the Better"), L27&lt;L26)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:W7 L9:W9 L11:W11 L13:W13 L15:W15 L17:W17 L19:W19 L21:W21 L23:W23 M27:W27 L29:W29 L31:W31 L33:W33 N35 Q35 T35:W35 O37 S37 U37:W37">
+    <cfRule type="expression" dxfId="62" priority="74">
+      <formula>AND(OR($H6="Lower the better", $H6="Lower the better"), L7&gt; L6)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="79">
-      <formula>AND(OR($H26="Lower the better", $H26="Lower the Better"), L27&lt;=L26)</formula>
+    <cfRule type="expression" dxfId="61" priority="247">
+      <formula>AND(OR($H6="Lower the better", $H6= "Lower the Better"), L7 &lt;= L6)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="78">
-      <formula>AND(OR($H26="Lower the better", $H26="Lower the Better"), L27&gt;L26)</formula>
+    <cfRule type="expression" dxfId="60" priority="248">
+      <formula>AND(OR($H6="Higher the better", $H6="Higher the Better"), L7 &lt; L6)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="59" priority="249">
+      <formula xml:space="preserve"> AND(OR($H6="Higher the better", $H6="Higher the Better"), L7&gt;= L6)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L7:W7 L9:W9 L11:W11 L13:W13 L15:W15 L17:W17 L19:W19 L21:W21 L23:W23 M27:W27 L29:W29 L31:W31 L33:W33 N35 Q35 T35:W35 O37 S37:W37">
-    <cfRule type="expression" dxfId="62" priority="249">
-      <formula xml:space="preserve"> AND(OR($H6="Higher the better", $H6="Higher the Better"), L7&gt;= L6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="61" priority="74">
-      <formula>AND(OR($H6="Lower the better", $H6="Lower the better"), L7&gt; L6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="60" priority="247">
-      <formula>AND(OR($H6="Lower the better", $H6= "Lower the Better"), L7 &lt;= L6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="59" priority="248">
-      <formula>AND(OR($H6="Higher the better", $H6="Higher the Better"), L7 &lt; L6)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L23:W27 L7:W7 L9:W9 L11:W11 L13:W13 L15:W15 L17:W17 L19:W19 L21:W21 L29:W29 L31:W31 L33:W33 N35 Q35 T35:W35 O37 S37:W37">
+  <conditionalFormatting sqref="L7:W7 L9:W9 L11:W11 L13:W13 L15:W15 L17:W17 L19:W19 L21:W21 L29:W29 L31:W31 L33:W33 N35 Q35 T35:W35 O37 S37 L23:W27 U37:W37">
     <cfRule type="containsBlanks" dxfId="58" priority="245">
       <formula>LEN(TRIM(L7))=0</formula>
     </cfRule>
@@ -12768,185 +12780,185 @@
     <cfRule type="containsBlanks" dxfId="56" priority="173">
       <formula>LEN(TRIM(L46))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="177">
-      <formula>AND(OR($H45="Higher the better", $H45="Higher the Better"), L46&lt;L45)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="54" priority="175">
+    <cfRule type="expression" dxfId="55" priority="175">
       <formula>AND(OR($H45="Lower the better", $H45="Lower the Better"), L46&gt;L45)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="176">
+    <cfRule type="expression" dxfId="54" priority="176">
       <formula>AND(OR($H45="Lower the better", $H45="Lower the Better"), L46&lt;=L45)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="53" priority="177">
+      <formula>AND(OR($H45="Higher the better", $H45="Higher the Better"), L46&lt;L45)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="52" priority="178" stopIfTrue="1">
       <formula>AND(OR($H45="Higher the better", $H45="Higher the Better"), L46&gt;=L45)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L52:W52">
-    <cfRule type="expression" dxfId="51" priority="107">
-      <formula>AND(OR($H51="Higher the better", $H51="Higher the Better"), L52&lt;L51)</formula>
+    <cfRule type="containsBlanks" dxfId="51" priority="104">
+      <formula>LEN(TRIM(L52))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="106">
+    <cfRule type="expression" dxfId="50" priority="105">
+      <formula>AND(OR($H51="Lower the better", $H51="Lower the Better"), L52&gt;L51)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="106">
       <formula>AND(OR($H51="Lower the better", $H51="Lower the Better"), L52&lt;=L51)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="49" priority="104">
-      <formula>LEN(TRIM(L52))=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="48" priority="105">
-      <formula>AND(OR($H51="Lower the better", $H51="Lower the Better"), L52&gt;L51)</formula>
+    <cfRule type="expression" dxfId="48" priority="107">
+      <formula>AND(OR($H51="Higher the better", $H51="Higher the Better"), L52&lt;L51)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="47" priority="108" stopIfTrue="1">
       <formula>AND(OR($H51="Higher the better", $H51="Higher the Better"), L52&gt;=L51)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N25 T25 W25 L42:W42">
-    <cfRule type="expression" dxfId="46" priority="71" stopIfTrue="1">
-      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), L25&gt;=L24)</formula>
+  <conditionalFormatting sqref="N25 W25 L42:W42">
+    <cfRule type="containsBlanks" dxfId="46" priority="67">
+      <formula>LEN(TRIM(L25))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="70">
+    <cfRule type="expression" dxfId="45" priority="68">
+      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), L25&gt;L24)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="69">
+      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), L25&lt;=L24)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="70">
       <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), L25&lt;L24)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="68">
-      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), L25&gt;L24)</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="43" priority="67">
-      <formula>LEN(TRIM(L25))=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="69">
-      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), L25&lt;=L24)</formula>
+    <cfRule type="expression" dxfId="42" priority="71" stopIfTrue="1">
+      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), L25&gt;=L24)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N25">
-    <cfRule type="expression" dxfId="41" priority="18">
-      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&lt;=N24)</formula>
+    <cfRule type="containsBlanks" dxfId="41" priority="16">
+      <formula>LEN(TRIM(N25))=0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="40" priority="17">
       <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&gt;N24)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="39" priority="16">
+    <cfRule type="expression" dxfId="39" priority="18">
+      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&lt;=N24)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="19">
+      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&lt;N24)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="20" stopIfTrue="1">
+      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&gt;=N24)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="36" priority="21">
       <formula>LEN(TRIM(N25))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="25" stopIfTrue="1">
-      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&gt;=N24)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="37" priority="22">
+    <cfRule type="expression" dxfId="35" priority="22">
       <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&gt;N24)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="24">
+    <cfRule type="expression" dxfId="34" priority="23">
+      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&lt;=N24)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="33" priority="24">
       <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&lt;N24)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="35" priority="21">
-      <formula>LEN(TRIM(N25))=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="32" priority="25" stopIfTrue="1">
       <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&gt;=N24)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="33" priority="23">
-      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), N25&lt;=N24)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="32" priority="19">
-      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), N25&lt;N24)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N44">
-    <cfRule type="expression" dxfId="31" priority="65">
+    <cfRule type="containsBlanks" dxfId="31" priority="62">
+      <formula>LEN(TRIM(N44))=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="30" priority="63">
+      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), N44&gt;N43)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="29" priority="64">
+      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), N44&lt;=N43)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="65">
       <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), N44&lt;N43)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="66" stopIfTrue="1">
       <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), N44&gt;=N43)</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="29" priority="62">
-      <formula>LEN(TRIM(N44))=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="63">
-      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), N44&gt;N43)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="64">
-      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), N44&lt;=N43)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q25">
-    <cfRule type="expression" dxfId="26" priority="30" stopIfTrue="1">
-      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), Q25&gt;=Q24)</formula>
+    <cfRule type="containsBlanks" dxfId="26" priority="26">
+      <formula>LEN(TRIM(Q25))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="29">
-      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), Q25&lt;Q24)</formula>
+    <cfRule type="expression" dxfId="25" priority="27">
+      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), Q25&gt;Q24)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="24" priority="28">
       <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), Q25&lt;=Q24)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="27">
-      <formula>AND(OR($H24="Lower the better", $H24="Lower the Better"), Q25&gt;Q24)</formula>
+    <cfRule type="expression" dxfId="23" priority="29">
+      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), Q25&lt;Q24)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="22" priority="26">
-      <formula>LEN(TRIM(Q25))=0</formula>
+    <cfRule type="expression" dxfId="22" priority="30" stopIfTrue="1">
+      <formula>AND(OR($H24="Higher the better", $H24="Higher the Better"), Q25&gt;=Q24)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q37">
-    <cfRule type="expression" dxfId="21" priority="10">
-      <formula xml:space="preserve"> AND(OR($H36="Higher the better", $H36="Higher the Better"), Q37&gt;= Q36)</formula>
+    <cfRule type="expression" dxfId="21" priority="6">
+      <formula>AND(OR($H36="Lower the better", $H36="Lower the better"), Q37&gt; Q36)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="9">
-      <formula>AND(OR($H36="Higher the better", $H36="Higher the Better"), Q37 &lt; Q36)</formula>
+    <cfRule type="containsBlanks" dxfId="20" priority="7">
+      <formula>LEN(TRIM(Q37))=0</formula>
     </cfRule>
     <cfRule type="expression" dxfId="19" priority="8">
       <formula>AND(OR($H36="Lower the better", $H36= "Lower the Better"), Q37 &lt;= Q36)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="6">
-      <formula>AND(OR($H36="Lower the better", $H36="Lower the better"), Q37&gt; Q36)</formula>
+    <cfRule type="expression" dxfId="18" priority="9">
+      <formula>AND(OR($H36="Higher the better", $H36="Higher the Better"), Q37 &lt; Q36)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="17" priority="7">
-      <formula>LEN(TRIM(Q37))=0</formula>
+    <cfRule type="expression" dxfId="17" priority="10">
+      <formula xml:space="preserve"> AND(OR($H36="Higher the better", $H36="Higher the Better"), Q37&gt;= Q36)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q44">
-    <cfRule type="expression" dxfId="16" priority="15" stopIfTrue="1">
-      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), Q44&gt;=Q43)</formula>
+    <cfRule type="containsBlanks" dxfId="16" priority="11">
+      <formula>LEN(TRIM(Q44))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="14">
-      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), Q44&lt;Q43)</formula>
+    <cfRule type="expression" dxfId="15" priority="12">
+      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), Q44&gt;Q43)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="14" priority="13">
       <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), Q44&lt;=Q43)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="12">
-      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), Q44&gt;Q43)</formula>
+    <cfRule type="expression" dxfId="13" priority="14">
+      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), Q44&lt;Q43)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="12" priority="11">
-      <formula>LEN(TRIM(Q44))=0</formula>
+    <cfRule type="expression" dxfId="12" priority="15" stopIfTrue="1">
+      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), Q44&gt;=Q43)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T44">
-    <cfRule type="expression" dxfId="11" priority="56" stopIfTrue="1">
-      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), T44&gt;=T43)</formula>
+    <cfRule type="containsBlanks" dxfId="11" priority="52">
+      <formula>LEN(TRIM(T44))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="55">
-      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), T44&lt;T43)</formula>
+    <cfRule type="expression" dxfId="10" priority="53">
+      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), T44&gt;T43)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="9" priority="54">
       <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), T44&lt;=T43)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="53">
-      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), T44&gt;T43)</formula>
+    <cfRule type="expression" dxfId="8" priority="55">
+      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), T44&lt;T43)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="7" priority="52">
-      <formula>LEN(TRIM(T44))=0</formula>
+    <cfRule type="expression" dxfId="7" priority="56" stopIfTrue="1">
+      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), T44&gt;=T43)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W44">
-    <cfRule type="expression" dxfId="6" priority="48">
+    <cfRule type="containsBlanks" dxfId="6" priority="47">
+      <formula>LEN(TRIM(W44))=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="48">
       <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), W44&gt;W43)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="5" priority="47">
-      <formula>LEN(TRIM(W44))=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="51" stopIfTrue="1">
-      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), W44&gt;=W43)</formula>
+    <cfRule type="expression" dxfId="4" priority="49">
+      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), W44&lt;=W43)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="3" priority="50">
       <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), W44&lt;W43)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="49">
-      <formula>AND(OR($H43="Lower the better", $H43="Lower the Better"), W44&lt;=W43)</formula>
+    <cfRule type="expression" dxfId="2" priority="51" stopIfTrue="1">
+      <formula>AND(OR($H43="Higher the better", $H43="Higher the Better"), W44&gt;=W43)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA47">
@@ -13155,40 +13167,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F096517C-598E-4E6D-B017-32F081EE1644}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{497B9C89-7047-44E4-9E7C-8AF16D1DE759}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B59988E5-FE96-444B-A770-A47DB401478A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B59988E5-FE96-444B-A770-A47DB401478A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4496F7DA-3E04-4F13-B9D0-FE26D9FB8ABD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4496F7DA-3E04-4F13-B9D0-FE26D9FB8ABD}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7094BB51-7951-4F88-97F3-C0EC6D9471D8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f5a961e1-edc1-4f62-8655-e8a46ef79e5c"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="68108f69-118e-4385-83b3-00743b1bf54c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7094BB51-7951-4F88-97F3-C0EC6D9471D8}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>